<commit_message>
[master] updated disk layout
</commit_message>
<xml_diff>
--- a/res/Disk layout.xlsx
+++ b/res/Disk layout.xlsx
@@ -47,7 +47,7 @@
         <rFont val="Arial"/>
         <color rgb="FFF3F3F3"/>
       </rPr>
-      <t xml:space="preserve">0.5 KB — 40 KB
+      <t xml:space="preserve">0.5 KB — 64 KB
 </t>
     </r>
     <r>
@@ -65,7 +65,7 @@
 ›boot›stage2.bin</t>
   </si>
   <si>
-    <t>40 KB</t>
+    <t>64 KB</t>
   </si>
   <si>
     <r>
@@ -73,7 +73,7 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t xml:space="preserve">40 KB — 10.6 MB
+      <t xml:space="preserve">64 KB — 10.6 MB
 </t>
     </r>
     <r>
@@ -99,7 +99,7 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t xml:space="preserve">10.6 MB — 12 MB
+      <t xml:space="preserve">10.6 MB — 11.6 MB
 </t>
     </r>
     <r>
@@ -117,7 +117,7 @@
 ›boot›kernel</t>
   </si>
   <si>
-    <t>12 MB</t>
+    <t>11.6 MB</t>
   </si>
   <si>
     <r>
@@ -125,7 +125,7 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t xml:space="preserve">12 MB — 
+      <t xml:space="preserve">11.6 MB — 
 </t>
     </r>
     <r>

</xml_diff>